<commit_message>
Re-run Respondent Bot on S01 after the output folder change
</commit_message>
<xml_diff>
--- a/out/S01_campus_cafeteria_experience/agent4/agent4_results.xlsx
+++ b/out/S01_campus_cafeteria_experience/agent4/agent4_results.xlsx
@@ -521,7 +521,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Survey id 318675, run 05 Oct 2026 00:37. The bot filled the survey as a respondent would and recorded what it saw. What a failure means is Agent 5's call.</t>
+          <t>Survey id 362829, run 11 Oct 2026 10:26. The bot filled the survey as a respondent would and recorded what it saw. What a failure means is Agent 5's call.</t>
         </is>
       </c>
     </row>
@@ -3390,7 +3390,7 @@
       </c>
       <c r="E2" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q708</t>
+          <t>LimeSurvey calls this question Q788</t>
         </is>
       </c>
     </row>
@@ -3436,7 +3436,7 @@
       </c>
       <c r="E4" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q709</t>
+          <t>LimeSurvey calls this question Q789</t>
         </is>
       </c>
     </row>
@@ -3482,7 +3482,7 @@
       </c>
       <c r="E6" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q710</t>
+          <t>LimeSurvey calls this question Q790</t>
         </is>
       </c>
     </row>
@@ -3528,7 +3528,7 @@
       </c>
       <c r="E8" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q711</t>
+          <t>LimeSurvey calls this question Q791</t>
         </is>
       </c>
     </row>
@@ -3574,7 +3574,7 @@
       </c>
       <c r="E10" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q712</t>
+          <t>LimeSurvey calls this question Q792</t>
         </is>
       </c>
     </row>
@@ -3620,7 +3620,7 @@
       </c>
       <c r="E12" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q713</t>
+          <t>LimeSurvey calls this question Q793</t>
         </is>
       </c>
     </row>
@@ -3666,7 +3666,7 @@
       </c>
       <c r="E14" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q714</t>
+          <t>LimeSurvey calls this question Q794</t>
         </is>
       </c>
     </row>
@@ -3712,7 +3712,7 @@
       </c>
       <c r="E16" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q715</t>
+          <t>LimeSurvey calls this question Q795</t>
         </is>
       </c>
     </row>
@@ -3758,7 +3758,7 @@
       </c>
       <c r="E18" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q716</t>
+          <t>LimeSurvey calls this question Q796</t>
         </is>
       </c>
     </row>
@@ -3850,7 +3850,7 @@
       </c>
       <c r="E22" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q708</t>
+          <t>LimeSurvey calls this question Q788</t>
         </is>
       </c>
     </row>
@@ -3896,7 +3896,7 @@
       </c>
       <c r="E24" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q708</t>
+          <t>LimeSurvey calls this question Q788</t>
         </is>
       </c>
     </row>
@@ -3942,7 +3942,7 @@
       </c>
       <c r="E26" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q709</t>
+          <t>LimeSurvey calls this question Q789</t>
         </is>
       </c>
     </row>
@@ -3988,7 +3988,7 @@
       </c>
       <c r="E28" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q710</t>
+          <t>LimeSurvey calls this question Q790</t>
         </is>
       </c>
     </row>
@@ -4034,7 +4034,7 @@
       </c>
       <c r="E30" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q711</t>
+          <t>LimeSurvey calls this question Q791</t>
         </is>
       </c>
     </row>
@@ -4080,7 +4080,7 @@
       </c>
       <c r="E32" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q712</t>
+          <t>LimeSurvey calls this question Q792</t>
         </is>
       </c>
     </row>
@@ -4126,7 +4126,7 @@
       </c>
       <c r="E34" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q713</t>
+          <t>LimeSurvey calls this question Q793</t>
         </is>
       </c>
     </row>
@@ -4172,7 +4172,7 @@
       </c>
       <c r="E36" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q714</t>
+          <t>LimeSurvey calls this question Q794</t>
         </is>
       </c>
     </row>
@@ -4218,7 +4218,7 @@
       </c>
       <c r="E38" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q715</t>
+          <t>LimeSurvey calls this question Q795</t>
         </is>
       </c>
     </row>
@@ -4264,7 +4264,7 @@
       </c>
       <c r="E40" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q716</t>
+          <t>LimeSurvey calls this question Q796</t>
         </is>
       </c>
     </row>
@@ -4310,7 +4310,7 @@
       </c>
       <c r="E42" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q708</t>
+          <t>LimeSurvey calls this question Q788</t>
         </is>
       </c>
     </row>
@@ -4402,7 +4402,7 @@
       </c>
       <c r="E46" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q708</t>
+          <t>LimeSurvey calls this question Q788</t>
         </is>
       </c>
     </row>
@@ -4448,7 +4448,7 @@
       </c>
       <c r="E48" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q709</t>
+          <t>LimeSurvey calls this question Q789</t>
         </is>
       </c>
     </row>
@@ -4494,7 +4494,7 @@
       </c>
       <c r="E50" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q708</t>
+          <t>LimeSurvey calls this question Q788</t>
         </is>
       </c>
     </row>
@@ -4540,7 +4540,7 @@
       </c>
       <c r="E52" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q709</t>
+          <t>LimeSurvey calls this question Q789</t>
         </is>
       </c>
     </row>
@@ -4586,7 +4586,7 @@
       </c>
       <c r="E54" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q710</t>
+          <t>LimeSurvey calls this question Q790</t>
         </is>
       </c>
     </row>
@@ -4632,7 +4632,7 @@
       </c>
       <c r="E56" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q711</t>
+          <t>LimeSurvey calls this question Q791</t>
         </is>
       </c>
     </row>
@@ -4678,7 +4678,7 @@
       </c>
       <c r="E58" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q712</t>
+          <t>LimeSurvey calls this question Q792</t>
         </is>
       </c>
     </row>
@@ -4724,7 +4724,7 @@
       </c>
       <c r="E60" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q713</t>
+          <t>LimeSurvey calls this question Q793</t>
         </is>
       </c>
     </row>
@@ -4770,7 +4770,7 @@
       </c>
       <c r="E62" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q714</t>
+          <t>LimeSurvey calls this question Q794</t>
         </is>
       </c>
     </row>
@@ -4816,7 +4816,7 @@
       </c>
       <c r="E64" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q715</t>
+          <t>LimeSurvey calls this question Q795</t>
         </is>
       </c>
     </row>
@@ -4862,7 +4862,7 @@
       </c>
       <c r="E66" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q716</t>
+          <t>LimeSurvey calls this question Q796</t>
         </is>
       </c>
     </row>
@@ -4908,7 +4908,7 @@
       </c>
       <c r="E68" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q708</t>
+          <t>LimeSurvey calls this question Q788</t>
         </is>
       </c>
     </row>
@@ -4954,7 +4954,7 @@
       </c>
       <c r="E70" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q709</t>
+          <t>LimeSurvey calls this question Q789</t>
         </is>
       </c>
     </row>
@@ -5046,7 +5046,7 @@
       </c>
       <c r="E74" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q708</t>
+          <t>LimeSurvey calls this question Q788</t>
         </is>
       </c>
     </row>
@@ -5092,7 +5092,7 @@
       </c>
       <c r="E76" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q709</t>
+          <t>LimeSurvey calls this question Q789</t>
         </is>
       </c>
     </row>
@@ -5138,7 +5138,7 @@
       </c>
       <c r="E78" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q710</t>
+          <t>LimeSurvey calls this question Q790</t>
         </is>
       </c>
     </row>
@@ -5184,7 +5184,7 @@
       </c>
       <c r="E80" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q711</t>
+          <t>LimeSurvey calls this question Q791</t>
         </is>
       </c>
     </row>
@@ -5230,7 +5230,7 @@
       </c>
       <c r="E82" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q712</t>
+          <t>LimeSurvey calls this question Q792</t>
         </is>
       </c>
     </row>
@@ -5276,7 +5276,7 @@
       </c>
       <c r="E84" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q713</t>
+          <t>LimeSurvey calls this question Q793</t>
         </is>
       </c>
     </row>
@@ -5322,7 +5322,7 @@
       </c>
       <c r="E86" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q714</t>
+          <t>LimeSurvey calls this question Q794</t>
         </is>
       </c>
     </row>
@@ -5368,7 +5368,7 @@
       </c>
       <c r="E88" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q715</t>
+          <t>LimeSurvey calls this question Q795</t>
         </is>
       </c>
     </row>
@@ -5414,7 +5414,7 @@
       </c>
       <c r="E90" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q716</t>
+          <t>LimeSurvey calls this question Q796</t>
         </is>
       </c>
     </row>
@@ -5460,7 +5460,7 @@
       </c>
       <c r="E92" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q708</t>
+          <t>LimeSurvey calls this question Q788</t>
         </is>
       </c>
     </row>
@@ -5506,7 +5506,7 @@
       </c>
       <c r="E94" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q709</t>
+          <t>LimeSurvey calls this question Q789</t>
         </is>
       </c>
     </row>
@@ -5552,7 +5552,7 @@
       </c>
       <c r="E96" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q710</t>
+          <t>LimeSurvey calls this question Q790</t>
         </is>
       </c>
     </row>
@@ -5644,7 +5644,7 @@
       </c>
       <c r="E100" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q708</t>
+          <t>LimeSurvey calls this question Q788</t>
         </is>
       </c>
     </row>
@@ -5690,7 +5690,7 @@
       </c>
       <c r="E102" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q709</t>
+          <t>LimeSurvey calls this question Q789</t>
         </is>
       </c>
     </row>
@@ -5736,7 +5736,7 @@
       </c>
       <c r="E104" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q710</t>
+          <t>LimeSurvey calls this question Q790</t>
         </is>
       </c>
     </row>
@@ -5782,7 +5782,7 @@
       </c>
       <c r="E106" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q711</t>
+          <t>LimeSurvey calls this question Q791</t>
         </is>
       </c>
     </row>
@@ -5828,7 +5828,7 @@
       </c>
       <c r="E108" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q712</t>
+          <t>LimeSurvey calls this question Q792</t>
         </is>
       </c>
     </row>
@@ -5874,7 +5874,7 @@
       </c>
       <c r="E110" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q713</t>
+          <t>LimeSurvey calls this question Q793</t>
         </is>
       </c>
     </row>
@@ -5920,7 +5920,7 @@
       </c>
       <c r="E112" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q714</t>
+          <t>LimeSurvey calls this question Q794</t>
         </is>
       </c>
     </row>
@@ -5966,7 +5966,7 @@
       </c>
       <c r="E114" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q715</t>
+          <t>LimeSurvey calls this question Q795</t>
         </is>
       </c>
     </row>
@@ -6012,7 +6012,7 @@
       </c>
       <c r="E116" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q716</t>
+          <t>LimeSurvey calls this question Q796</t>
         </is>
       </c>
     </row>
@@ -6058,7 +6058,7 @@
       </c>
       <c r="E118" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q708</t>
+          <t>LimeSurvey calls this question Q788</t>
         </is>
       </c>
     </row>
@@ -6104,7 +6104,7 @@
       </c>
       <c r="E120" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q709</t>
+          <t>LimeSurvey calls this question Q789</t>
         </is>
       </c>
     </row>
@@ -6150,7 +6150,7 @@
       </c>
       <c r="E122" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q710</t>
+          <t>LimeSurvey calls this question Q790</t>
         </is>
       </c>
     </row>
@@ -6196,7 +6196,7 @@
       </c>
       <c r="E124" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q711</t>
+          <t>LimeSurvey calls this question Q791</t>
         </is>
       </c>
     </row>
@@ -6288,7 +6288,7 @@
       </c>
       <c r="E128" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q708</t>
+          <t>LimeSurvey calls this question Q788</t>
         </is>
       </c>
     </row>
@@ -6334,7 +6334,7 @@
       </c>
       <c r="E130" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q709</t>
+          <t>LimeSurvey calls this question Q789</t>
         </is>
       </c>
     </row>
@@ -6380,7 +6380,7 @@
       </c>
       <c r="E132" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q710</t>
+          <t>LimeSurvey calls this question Q790</t>
         </is>
       </c>
     </row>
@@ -6426,7 +6426,7 @@
       </c>
       <c r="E134" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q711</t>
+          <t>LimeSurvey calls this question Q791</t>
         </is>
       </c>
     </row>
@@ -6472,7 +6472,7 @@
       </c>
       <c r="E136" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q712</t>
+          <t>LimeSurvey calls this question Q792</t>
         </is>
       </c>
     </row>
@@ -6518,7 +6518,7 @@
       </c>
       <c r="E138" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q713</t>
+          <t>LimeSurvey calls this question Q793</t>
         </is>
       </c>
     </row>
@@ -6564,7 +6564,7 @@
       </c>
       <c r="E140" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q714</t>
+          <t>LimeSurvey calls this question Q794</t>
         </is>
       </c>
     </row>
@@ -6610,7 +6610,7 @@
       </c>
       <c r="E142" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q715</t>
+          <t>LimeSurvey calls this question Q795</t>
         </is>
       </c>
     </row>
@@ -6656,7 +6656,7 @@
       </c>
       <c r="E144" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q716</t>
+          <t>LimeSurvey calls this question Q796</t>
         </is>
       </c>
     </row>
@@ -6702,7 +6702,7 @@
       </c>
       <c r="E146" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q708</t>
+          <t>LimeSurvey calls this question Q788</t>
         </is>
       </c>
     </row>
@@ -6748,7 +6748,7 @@
       </c>
       <c r="E148" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q709</t>
+          <t>LimeSurvey calls this question Q789</t>
         </is>
       </c>
     </row>
@@ -6794,7 +6794,7 @@
       </c>
       <c r="E150" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q710</t>
+          <t>LimeSurvey calls this question Q790</t>
         </is>
       </c>
     </row>
@@ -6840,7 +6840,7 @@
       </c>
       <c r="E152" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q711</t>
+          <t>LimeSurvey calls this question Q791</t>
         </is>
       </c>
     </row>
@@ -6886,7 +6886,7 @@
       </c>
       <c r="E154" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q712</t>
+          <t>LimeSurvey calls this question Q792</t>
         </is>
       </c>
     </row>
@@ -6932,7 +6932,7 @@
       </c>
       <c r="E156" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q713</t>
+          <t>LimeSurvey calls this question Q793</t>
         </is>
       </c>
     </row>
@@ -6978,7 +6978,7 @@
       </c>
       <c r="E158" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q708</t>
+          <t>LimeSurvey calls this question Q788</t>
         </is>
       </c>
     </row>
@@ -7024,7 +7024,7 @@
       </c>
       <c r="E160" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q709</t>
+          <t>LimeSurvey calls this question Q789</t>
         </is>
       </c>
     </row>
@@ -7070,7 +7070,7 @@
       </c>
       <c r="E162" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q710</t>
+          <t>LimeSurvey calls this question Q790</t>
         </is>
       </c>
     </row>
@@ -7116,7 +7116,7 @@
       </c>
       <c r="E164" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q711</t>
+          <t>LimeSurvey calls this question Q791</t>
         </is>
       </c>
     </row>
@@ -7162,7 +7162,7 @@
       </c>
       <c r="E166" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q712</t>
+          <t>LimeSurvey calls this question Q792</t>
         </is>
       </c>
     </row>
@@ -7254,7 +7254,7 @@
       </c>
       <c r="E170" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q708</t>
+          <t>LimeSurvey calls this question Q788</t>
         </is>
       </c>
     </row>
@@ -7300,7 +7300,7 @@
       </c>
       <c r="E172" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q709</t>
+          <t>LimeSurvey calls this question Q789</t>
         </is>
       </c>
     </row>
@@ -7346,7 +7346,7 @@
       </c>
       <c r="E174" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q710</t>
+          <t>LimeSurvey calls this question Q790</t>
         </is>
       </c>
     </row>
@@ -7392,7 +7392,7 @@
       </c>
       <c r="E176" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q711</t>
+          <t>LimeSurvey calls this question Q791</t>
         </is>
       </c>
     </row>
@@ -7438,7 +7438,7 @@
       </c>
       <c r="E178" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q712</t>
+          <t>LimeSurvey calls this question Q792</t>
         </is>
       </c>
     </row>
@@ -7530,7 +7530,7 @@
       </c>
       <c r="E182" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q708</t>
+          <t>LimeSurvey calls this question Q788</t>
         </is>
       </c>
     </row>
@@ -7576,7 +7576,7 @@
       </c>
       <c r="E184" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q709</t>
+          <t>LimeSurvey calls this question Q789</t>
         </is>
       </c>
     </row>
@@ -7622,7 +7622,7 @@
       </c>
       <c r="E186" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q710</t>
+          <t>LimeSurvey calls this question Q790</t>
         </is>
       </c>
     </row>
@@ -7668,7 +7668,7 @@
       </c>
       <c r="E188" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q711</t>
+          <t>LimeSurvey calls this question Q791</t>
         </is>
       </c>
     </row>
@@ -7714,7 +7714,7 @@
       </c>
       <c r="E190" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q712</t>
+          <t>LimeSurvey calls this question Q792</t>
         </is>
       </c>
     </row>
@@ -7760,7 +7760,7 @@
       </c>
       <c r="E192" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q713</t>
+          <t>LimeSurvey calls this question Q793</t>
         </is>
       </c>
     </row>
@@ -7806,7 +7806,7 @@
       </c>
       <c r="E194" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q714</t>
+          <t>LimeSurvey calls this question Q794</t>
         </is>
       </c>
     </row>
@@ -7852,7 +7852,7 @@
       </c>
       <c r="E196" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q715</t>
+          <t>LimeSurvey calls this question Q795</t>
         </is>
       </c>
     </row>
@@ -7898,7 +7898,7 @@
       </c>
       <c r="E198" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q716</t>
+          <t>LimeSurvey calls this question Q796</t>
         </is>
       </c>
     </row>
@@ -7944,7 +7944,7 @@
       </c>
       <c r="E200" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q708</t>
+          <t>LimeSurvey calls this question Q788</t>
         </is>
       </c>
     </row>
@@ -7990,7 +7990,7 @@
       </c>
       <c r="E202" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q709</t>
+          <t>LimeSurvey calls this question Q789</t>
         </is>
       </c>
     </row>
@@ -8036,7 +8036,7 @@
       </c>
       <c r="E204" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q710</t>
+          <t>LimeSurvey calls this question Q790</t>
         </is>
       </c>
     </row>
@@ -8082,7 +8082,7 @@
       </c>
       <c r="E206" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q711</t>
+          <t>LimeSurvey calls this question Q791</t>
         </is>
       </c>
     </row>
@@ -8128,7 +8128,7 @@
       </c>
       <c r="E208" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q712</t>
+          <t>LimeSurvey calls this question Q792</t>
         </is>
       </c>
     </row>
@@ -8174,7 +8174,7 @@
       </c>
       <c r="E210" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q713</t>
+          <t>LimeSurvey calls this question Q793</t>
         </is>
       </c>
     </row>
@@ -8220,7 +8220,7 @@
       </c>
       <c r="E212" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q714</t>
+          <t>LimeSurvey calls this question Q794</t>
         </is>
       </c>
     </row>
@@ -8266,7 +8266,7 @@
       </c>
       <c r="E214" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q708</t>
+          <t>LimeSurvey calls this question Q788</t>
         </is>
       </c>
     </row>
@@ -8312,7 +8312,7 @@
       </c>
       <c r="E216" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q709</t>
+          <t>LimeSurvey calls this question Q789</t>
         </is>
       </c>
     </row>
@@ -8358,7 +8358,7 @@
       </c>
       <c r="E218" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q710</t>
+          <t>LimeSurvey calls this question Q790</t>
         </is>
       </c>
     </row>
@@ -8404,7 +8404,7 @@
       </c>
       <c r="E220" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q711</t>
+          <t>LimeSurvey calls this question Q791</t>
         </is>
       </c>
     </row>
@@ -8450,7 +8450,7 @@
       </c>
       <c r="E222" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q712</t>
+          <t>LimeSurvey calls this question Q792</t>
         </is>
       </c>
     </row>
@@ -8496,7 +8496,7 @@
       </c>
       <c r="E224" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q713</t>
+          <t>LimeSurvey calls this question Q793</t>
         </is>
       </c>
     </row>
@@ -8542,7 +8542,7 @@
       </c>
       <c r="E226" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q714</t>
+          <t>LimeSurvey calls this question Q794</t>
         </is>
       </c>
     </row>
@@ -8588,7 +8588,7 @@
       </c>
       <c r="E228" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q708</t>
+          <t>LimeSurvey calls this question Q788</t>
         </is>
       </c>
     </row>
@@ -8634,7 +8634,7 @@
       </c>
       <c r="E230" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q709</t>
+          <t>LimeSurvey calls this question Q789</t>
         </is>
       </c>
     </row>
@@ -8680,7 +8680,7 @@
       </c>
       <c r="E232" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q710</t>
+          <t>LimeSurvey calls this question Q790</t>
         </is>
       </c>
     </row>
@@ -8726,7 +8726,7 @@
       </c>
       <c r="E234" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q711</t>
+          <t>LimeSurvey calls this question Q791</t>
         </is>
       </c>
     </row>
@@ -8772,7 +8772,7 @@
       </c>
       <c r="E236" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q712</t>
+          <t>LimeSurvey calls this question Q792</t>
         </is>
       </c>
     </row>
@@ -8818,7 +8818,7 @@
       </c>
       <c r="E238" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q713</t>
+          <t>LimeSurvey calls this question Q793</t>
         </is>
       </c>
     </row>
@@ -8910,7 +8910,7 @@
       </c>
       <c r="E242" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q708</t>
+          <t>LimeSurvey calls this question Q788</t>
         </is>
       </c>
     </row>
@@ -8956,7 +8956,7 @@
       </c>
       <c r="E244" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q709</t>
+          <t>LimeSurvey calls this question Q789</t>
         </is>
       </c>
     </row>
@@ -9002,7 +9002,7 @@
       </c>
       <c r="E246" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q710</t>
+          <t>LimeSurvey calls this question Q790</t>
         </is>
       </c>
     </row>
@@ -9048,7 +9048,7 @@
       </c>
       <c r="E248" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q711</t>
+          <t>LimeSurvey calls this question Q791</t>
         </is>
       </c>
     </row>
@@ -9094,7 +9094,7 @@
       </c>
       <c r="E250" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q712</t>
+          <t>LimeSurvey calls this question Q792</t>
         </is>
       </c>
     </row>
@@ -9140,7 +9140,7 @@
       </c>
       <c r="E252" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q713</t>
+          <t>LimeSurvey calls this question Q793</t>
         </is>
       </c>
     </row>
@@ -9186,7 +9186,7 @@
       </c>
       <c r="E254" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q714</t>
+          <t>LimeSurvey calls this question Q794</t>
         </is>
       </c>
     </row>
@@ -9232,7 +9232,7 @@
       </c>
       <c r="E256" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q715</t>
+          <t>LimeSurvey calls this question Q795</t>
         </is>
       </c>
     </row>
@@ -9278,7 +9278,7 @@
       </c>
       <c r="E258" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q716</t>
+          <t>LimeSurvey calls this question Q796</t>
         </is>
       </c>
     </row>
@@ -9324,7 +9324,7 @@
       </c>
       <c r="E260" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q708</t>
+          <t>LimeSurvey calls this question Q788</t>
         </is>
       </c>
     </row>
@@ -9370,7 +9370,7 @@
       </c>
       <c r="E262" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q709</t>
+          <t>LimeSurvey calls this question Q789</t>
         </is>
       </c>
     </row>
@@ -9416,7 +9416,7 @@
       </c>
       <c r="E264" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q710</t>
+          <t>LimeSurvey calls this question Q790</t>
         </is>
       </c>
     </row>
@@ -9462,7 +9462,7 @@
       </c>
       <c r="E266" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q711</t>
+          <t>LimeSurvey calls this question Q791</t>
         </is>
       </c>
     </row>
@@ -9508,7 +9508,7 @@
       </c>
       <c r="E268" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q712</t>
+          <t>LimeSurvey calls this question Q792</t>
         </is>
       </c>
     </row>
@@ -9554,7 +9554,7 @@
       </c>
       <c r="E270" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q713</t>
+          <t>LimeSurvey calls this question Q793</t>
         </is>
       </c>
     </row>
@@ -9600,7 +9600,7 @@
       </c>
       <c r="E272" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q714</t>
+          <t>LimeSurvey calls this question Q794</t>
         </is>
       </c>
     </row>
@@ -9646,7 +9646,7 @@
       </c>
       <c r="E274" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q715</t>
+          <t>LimeSurvey calls this question Q795</t>
         </is>
       </c>
     </row>
@@ -9692,7 +9692,7 @@
       </c>
       <c r="E276" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q708</t>
+          <t>LimeSurvey calls this question Q788</t>
         </is>
       </c>
     </row>
@@ -9738,7 +9738,7 @@
       </c>
       <c r="E278" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q709</t>
+          <t>LimeSurvey calls this question Q789</t>
         </is>
       </c>
     </row>
@@ -9784,7 +9784,7 @@
       </c>
       <c r="E280" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q710</t>
+          <t>LimeSurvey calls this question Q790</t>
         </is>
       </c>
     </row>
@@ -9830,7 +9830,7 @@
       </c>
       <c r="E282" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q711</t>
+          <t>LimeSurvey calls this question Q791</t>
         </is>
       </c>
     </row>
@@ -9876,7 +9876,7 @@
       </c>
       <c r="E284" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q712</t>
+          <t>LimeSurvey calls this question Q792</t>
         </is>
       </c>
     </row>
@@ -9922,7 +9922,7 @@
       </c>
       <c r="E286" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q713</t>
+          <t>LimeSurvey calls this question Q793</t>
         </is>
       </c>
     </row>
@@ -9968,7 +9968,7 @@
       </c>
       <c r="E288" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q714</t>
+          <t>LimeSurvey calls this question Q794</t>
         </is>
       </c>
     </row>
@@ -10014,7 +10014,7 @@
       </c>
       <c r="E290" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q708</t>
+          <t>LimeSurvey calls this question Q788</t>
         </is>
       </c>
     </row>
@@ -10060,7 +10060,7 @@
       </c>
       <c r="E292" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q709</t>
+          <t>LimeSurvey calls this question Q789</t>
         </is>
       </c>
     </row>
@@ -10106,7 +10106,7 @@
       </c>
       <c r="E294" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q710</t>
+          <t>LimeSurvey calls this question Q790</t>
         </is>
       </c>
     </row>
@@ -10152,7 +10152,7 @@
       </c>
       <c r="E296" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q711</t>
+          <t>LimeSurvey calls this question Q791</t>
         </is>
       </c>
     </row>
@@ -10198,7 +10198,7 @@
       </c>
       <c r="E298" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q712</t>
+          <t>LimeSurvey calls this question Q792</t>
         </is>
       </c>
     </row>
@@ -10244,7 +10244,7 @@
       </c>
       <c r="E300" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q713</t>
+          <t>LimeSurvey calls this question Q793</t>
         </is>
       </c>
     </row>
@@ -10290,7 +10290,7 @@
       </c>
       <c r="E302" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q714</t>
+          <t>LimeSurvey calls this question Q794</t>
         </is>
       </c>
     </row>
@@ -10336,7 +10336,7 @@
       </c>
       <c r="E304" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q715</t>
+          <t>LimeSurvey calls this question Q795</t>
         </is>
       </c>
     </row>
@@ -10382,7 +10382,7 @@
       </c>
       <c r="E306" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q708</t>
+          <t>LimeSurvey calls this question Q788</t>
         </is>
       </c>
     </row>
@@ -10428,7 +10428,7 @@
       </c>
       <c r="E308" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q709</t>
+          <t>LimeSurvey calls this question Q789</t>
         </is>
       </c>
     </row>
@@ -10474,7 +10474,7 @@
       </c>
       <c r="E310" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q710</t>
+          <t>LimeSurvey calls this question Q790</t>
         </is>
       </c>
     </row>
@@ -10520,7 +10520,7 @@
       </c>
       <c r="E312" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q711</t>
+          <t>LimeSurvey calls this question Q791</t>
         </is>
       </c>
     </row>
@@ -10566,7 +10566,7 @@
       </c>
       <c r="E314" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q712</t>
+          <t>LimeSurvey calls this question Q792</t>
         </is>
       </c>
     </row>
@@ -10612,7 +10612,7 @@
       </c>
       <c r="E316" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q713</t>
+          <t>LimeSurvey calls this question Q793</t>
         </is>
       </c>
     </row>
@@ -10658,7 +10658,7 @@
       </c>
       <c r="E318" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q714</t>
+          <t>LimeSurvey calls this question Q794</t>
         </is>
       </c>
     </row>
@@ -10704,7 +10704,7 @@
       </c>
       <c r="E320" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q715</t>
+          <t>LimeSurvey calls this question Q795</t>
         </is>
       </c>
     </row>
@@ -10750,7 +10750,7 @@
       </c>
       <c r="E322" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q708</t>
+          <t>LimeSurvey calls this question Q788</t>
         </is>
       </c>
     </row>
@@ -10796,7 +10796,7 @@
       </c>
       <c r="E324" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q709</t>
+          <t>LimeSurvey calls this question Q789</t>
         </is>
       </c>
     </row>
@@ -10842,7 +10842,7 @@
       </c>
       <c r="E326" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q710</t>
+          <t>LimeSurvey calls this question Q790</t>
         </is>
       </c>
     </row>
@@ -10888,7 +10888,7 @@
       </c>
       <c r="E328" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q711</t>
+          <t>LimeSurvey calls this question Q791</t>
         </is>
       </c>
     </row>
@@ -10934,7 +10934,7 @@
       </c>
       <c r="E330" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q712</t>
+          <t>LimeSurvey calls this question Q792</t>
         </is>
       </c>
     </row>
@@ -10980,7 +10980,7 @@
       </c>
       <c r="E332" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q713</t>
+          <t>LimeSurvey calls this question Q793</t>
         </is>
       </c>
     </row>
@@ -11026,7 +11026,7 @@
       </c>
       <c r="E334" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q714</t>
+          <t>LimeSurvey calls this question Q794</t>
         </is>
       </c>
     </row>
@@ -11118,7 +11118,7 @@
       </c>
       <c r="E338" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q708</t>
+          <t>LimeSurvey calls this question Q788</t>
         </is>
       </c>
     </row>
@@ -11164,7 +11164,7 @@
       </c>
       <c r="E340" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q709</t>
+          <t>LimeSurvey calls this question Q789</t>
         </is>
       </c>
     </row>
@@ -11210,7 +11210,7 @@
       </c>
       <c r="E342" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q710</t>
+          <t>LimeSurvey calls this question Q790</t>
         </is>
       </c>
     </row>
@@ -11256,7 +11256,7 @@
       </c>
       <c r="E344" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q711</t>
+          <t>LimeSurvey calls this question Q791</t>
         </is>
       </c>
     </row>
@@ -11302,7 +11302,7 @@
       </c>
       <c r="E346" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q712</t>
+          <t>LimeSurvey calls this question Q792</t>
         </is>
       </c>
     </row>
@@ -11348,7 +11348,7 @@
       </c>
       <c r="E348" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q713</t>
+          <t>LimeSurvey calls this question Q793</t>
         </is>
       </c>
     </row>
@@ -11394,7 +11394,7 @@
       </c>
       <c r="E350" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q714</t>
+          <t>LimeSurvey calls this question Q794</t>
         </is>
       </c>
     </row>
@@ -11440,7 +11440,7 @@
       </c>
       <c r="E352" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q715</t>
+          <t>LimeSurvey calls this question Q795</t>
         </is>
       </c>
     </row>
@@ -11486,7 +11486,7 @@
       </c>
       <c r="E354" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q708</t>
+          <t>LimeSurvey calls this question Q788</t>
         </is>
       </c>
     </row>
@@ -11532,7 +11532,7 @@
       </c>
       <c r="E356" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q709</t>
+          <t>LimeSurvey calls this question Q789</t>
         </is>
       </c>
     </row>
@@ -11578,7 +11578,7 @@
       </c>
       <c r="E358" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q710</t>
+          <t>LimeSurvey calls this question Q790</t>
         </is>
       </c>
     </row>
@@ -11624,7 +11624,7 @@
       </c>
       <c r="E360" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q711</t>
+          <t>LimeSurvey calls this question Q791</t>
         </is>
       </c>
     </row>
@@ -11670,7 +11670,7 @@
       </c>
       <c r="E362" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q712</t>
+          <t>LimeSurvey calls this question Q792</t>
         </is>
       </c>
     </row>
@@ -11716,7 +11716,7 @@
       </c>
       <c r="E364" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q713</t>
+          <t>LimeSurvey calls this question Q793</t>
         </is>
       </c>
     </row>
@@ -11762,7 +11762,7 @@
       </c>
       <c r="E366" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q714</t>
+          <t>LimeSurvey calls this question Q794</t>
         </is>
       </c>
     </row>
@@ -11808,7 +11808,7 @@
       </c>
       <c r="E368" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q715</t>
+          <t>LimeSurvey calls this question Q795</t>
         </is>
       </c>
     </row>
@@ -11854,7 +11854,7 @@
       </c>
       <c r="E370" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q708</t>
+          <t>LimeSurvey calls this question Q788</t>
         </is>
       </c>
     </row>
@@ -11900,7 +11900,7 @@
       </c>
       <c r="E372" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q709</t>
+          <t>LimeSurvey calls this question Q789</t>
         </is>
       </c>
     </row>
@@ -11946,7 +11946,7 @@
       </c>
       <c r="E374" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q710</t>
+          <t>LimeSurvey calls this question Q790</t>
         </is>
       </c>
     </row>
@@ -11992,7 +11992,7 @@
       </c>
       <c r="E376" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q711</t>
+          <t>LimeSurvey calls this question Q791</t>
         </is>
       </c>
     </row>
@@ -12038,7 +12038,7 @@
       </c>
       <c r="E378" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q712</t>
+          <t>LimeSurvey calls this question Q792</t>
         </is>
       </c>
     </row>
@@ -12084,7 +12084,7 @@
       </c>
       <c r="E380" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q713</t>
+          <t>LimeSurvey calls this question Q793</t>
         </is>
       </c>
     </row>
@@ -12130,7 +12130,7 @@
       </c>
       <c r="E382" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q714</t>
+          <t>LimeSurvey calls this question Q794</t>
         </is>
       </c>
     </row>
@@ -12176,7 +12176,7 @@
       </c>
       <c r="E384" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q715</t>
+          <t>LimeSurvey calls this question Q795</t>
         </is>
       </c>
     </row>
@@ -12222,7 +12222,7 @@
       </c>
       <c r="E386" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q708</t>
+          <t>LimeSurvey calls this question Q788</t>
         </is>
       </c>
     </row>
@@ -12268,7 +12268,7 @@
       </c>
       <c r="E388" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q709</t>
+          <t>LimeSurvey calls this question Q789</t>
         </is>
       </c>
     </row>
@@ -12314,7 +12314,7 @@
       </c>
       <c r="E390" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q710</t>
+          <t>LimeSurvey calls this question Q790</t>
         </is>
       </c>
     </row>
@@ -12360,7 +12360,7 @@
       </c>
       <c r="E392" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q711</t>
+          <t>LimeSurvey calls this question Q791</t>
         </is>
       </c>
     </row>
@@ -12406,7 +12406,7 @@
       </c>
       <c r="E394" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q712</t>
+          <t>LimeSurvey calls this question Q792</t>
         </is>
       </c>
     </row>
@@ -12452,7 +12452,7 @@
       </c>
       <c r="E396" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q713</t>
+          <t>LimeSurvey calls this question Q793</t>
         </is>
       </c>
     </row>
@@ -12498,7 +12498,7 @@
       </c>
       <c r="E398" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q714</t>
+          <t>LimeSurvey calls this question Q794</t>
         </is>
       </c>
     </row>
@@ -12544,7 +12544,7 @@
       </c>
       <c r="E400" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q715</t>
+          <t>LimeSurvey calls this question Q795</t>
         </is>
       </c>
     </row>
@@ -12590,7 +12590,7 @@
       </c>
       <c r="E402" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q708</t>
+          <t>LimeSurvey calls this question Q788</t>
         </is>
       </c>
     </row>
@@ -12636,7 +12636,7 @@
       </c>
       <c r="E404" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q709</t>
+          <t>LimeSurvey calls this question Q789</t>
         </is>
       </c>
     </row>
@@ -12682,7 +12682,7 @@
       </c>
       <c r="E406" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q710</t>
+          <t>LimeSurvey calls this question Q790</t>
         </is>
       </c>
     </row>
@@ -12728,7 +12728,7 @@
       </c>
       <c r="E408" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q711</t>
+          <t>LimeSurvey calls this question Q791</t>
         </is>
       </c>
     </row>
@@ -12774,7 +12774,7 @@
       </c>
       <c r="E410" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q712</t>
+          <t>LimeSurvey calls this question Q792</t>
         </is>
       </c>
     </row>
@@ -12820,7 +12820,7 @@
       </c>
       <c r="E412" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q713</t>
+          <t>LimeSurvey calls this question Q793</t>
         </is>
       </c>
     </row>
@@ -12866,7 +12866,7 @@
       </c>
       <c r="E414" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q714</t>
+          <t>LimeSurvey calls this question Q794</t>
         </is>
       </c>
     </row>
@@ -12912,7 +12912,7 @@
       </c>
       <c r="E416" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q715</t>
+          <t>LimeSurvey calls this question Q795</t>
         </is>
       </c>
     </row>
@@ -12958,7 +12958,7 @@
       </c>
       <c r="E418" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q708</t>
+          <t>LimeSurvey calls this question Q788</t>
         </is>
       </c>
     </row>
@@ -13004,7 +13004,7 @@
       </c>
       <c r="E420" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q709</t>
+          <t>LimeSurvey calls this question Q789</t>
         </is>
       </c>
     </row>
@@ -13050,7 +13050,7 @@
       </c>
       <c r="E422" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q710</t>
+          <t>LimeSurvey calls this question Q790</t>
         </is>
       </c>
     </row>
@@ -13096,7 +13096,7 @@
       </c>
       <c r="E424" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q711</t>
+          <t>LimeSurvey calls this question Q791</t>
         </is>
       </c>
     </row>
@@ -13142,7 +13142,7 @@
       </c>
       <c r="E426" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q712</t>
+          <t>LimeSurvey calls this question Q792</t>
         </is>
       </c>
     </row>
@@ -13188,7 +13188,7 @@
       </c>
       <c r="E428" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q713</t>
+          <t>LimeSurvey calls this question Q793</t>
         </is>
       </c>
     </row>
@@ -13234,7 +13234,7 @@
       </c>
       <c r="E430" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q714</t>
+          <t>LimeSurvey calls this question Q794</t>
         </is>
       </c>
     </row>
@@ -13280,7 +13280,7 @@
       </c>
       <c r="E432" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q715</t>
+          <t>LimeSurvey calls this question Q795</t>
         </is>
       </c>
     </row>
@@ -13326,7 +13326,7 @@
       </c>
       <c r="E434" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q716</t>
+          <t>LimeSurvey calls this question Q796</t>
         </is>
       </c>
     </row>
@@ -13372,7 +13372,7 @@
       </c>
       <c r="E436" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q708</t>
+          <t>LimeSurvey calls this question Q788</t>
         </is>
       </c>
     </row>
@@ -13418,7 +13418,7 @@
       </c>
       <c r="E438" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q709</t>
+          <t>LimeSurvey calls this question Q789</t>
         </is>
       </c>
     </row>
@@ -13464,7 +13464,7 @@
       </c>
       <c r="E440" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q710</t>
+          <t>LimeSurvey calls this question Q790</t>
         </is>
       </c>
     </row>
@@ -13510,7 +13510,7 @@
       </c>
       <c r="E442" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q711</t>
+          <t>LimeSurvey calls this question Q791</t>
         </is>
       </c>
     </row>
@@ -13556,7 +13556,7 @@
       </c>
       <c r="E444" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q712</t>
+          <t>LimeSurvey calls this question Q792</t>
         </is>
       </c>
     </row>
@@ -13602,7 +13602,7 @@
       </c>
       <c r="E446" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q713</t>
+          <t>LimeSurvey calls this question Q793</t>
         </is>
       </c>
     </row>
@@ -13648,7 +13648,7 @@
       </c>
       <c r="E448" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q714</t>
+          <t>LimeSurvey calls this question Q794</t>
         </is>
       </c>
     </row>
@@ -13694,7 +13694,7 @@
       </c>
       <c r="E450" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q715</t>
+          <t>LimeSurvey calls this question Q795</t>
         </is>
       </c>
     </row>
@@ -13786,7 +13786,7 @@
       </c>
       <c r="E454" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q708</t>
+          <t>LimeSurvey calls this question Q788</t>
         </is>
       </c>
     </row>
@@ -13832,7 +13832,7 @@
       </c>
       <c r="E456" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q709</t>
+          <t>LimeSurvey calls this question Q789</t>
         </is>
       </c>
     </row>
@@ -13878,7 +13878,7 @@
       </c>
       <c r="E458" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q710</t>
+          <t>LimeSurvey calls this question Q790</t>
         </is>
       </c>
     </row>
@@ -13924,7 +13924,7 @@
       </c>
       <c r="E460" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q711</t>
+          <t>LimeSurvey calls this question Q791</t>
         </is>
       </c>
     </row>
@@ -13970,7 +13970,7 @@
       </c>
       <c r="E462" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q712</t>
+          <t>LimeSurvey calls this question Q792</t>
         </is>
       </c>
     </row>
@@ -14016,7 +14016,7 @@
       </c>
       <c r="E464" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q713</t>
+          <t>LimeSurvey calls this question Q793</t>
         </is>
       </c>
     </row>
@@ -14062,7 +14062,7 @@
       </c>
       <c r="E466" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q714</t>
+          <t>LimeSurvey calls this question Q794</t>
         </is>
       </c>
     </row>
@@ -14108,7 +14108,7 @@
       </c>
       <c r="E468" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q715</t>
+          <t>LimeSurvey calls this question Q795</t>
         </is>
       </c>
     </row>
@@ -14154,7 +14154,7 @@
       </c>
       <c r="E470" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q716</t>
+          <t>LimeSurvey calls this question Q796</t>
         </is>
       </c>
     </row>
@@ -14200,7 +14200,7 @@
       </c>
       <c r="E472" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q708</t>
+          <t>LimeSurvey calls this question Q788</t>
         </is>
       </c>
     </row>
@@ -14246,7 +14246,7 @@
       </c>
       <c r="E474" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q709</t>
+          <t>LimeSurvey calls this question Q789</t>
         </is>
       </c>
     </row>
@@ -14292,7 +14292,7 @@
       </c>
       <c r="E476" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q710</t>
+          <t>LimeSurvey calls this question Q790</t>
         </is>
       </c>
     </row>
@@ -14338,7 +14338,7 @@
       </c>
       <c r="E478" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q711</t>
+          <t>LimeSurvey calls this question Q791</t>
         </is>
       </c>
     </row>
@@ -14384,7 +14384,7 @@
       </c>
       <c r="E480" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q712</t>
+          <t>LimeSurvey calls this question Q792</t>
         </is>
       </c>
     </row>
@@ -14430,7 +14430,7 @@
       </c>
       <c r="E482" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q713</t>
+          <t>LimeSurvey calls this question Q793</t>
         </is>
       </c>
     </row>
@@ -14476,7 +14476,7 @@
       </c>
       <c r="E484" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q714</t>
+          <t>LimeSurvey calls this question Q794</t>
         </is>
       </c>
     </row>
@@ -14522,7 +14522,7 @@
       </c>
       <c r="E486" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q715</t>
+          <t>LimeSurvey calls this question Q795</t>
         </is>
       </c>
     </row>
@@ -14568,7 +14568,7 @@
       </c>
       <c r="E488" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q716</t>
+          <t>LimeSurvey calls this question Q796</t>
         </is>
       </c>
     </row>
@@ -14614,7 +14614,7 @@
       </c>
       <c r="E490" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q717</t>
+          <t>LimeSurvey calls this question Q797</t>
         </is>
       </c>
     </row>
@@ -14660,7 +14660,7 @@
       </c>
       <c r="E492" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q708</t>
+          <t>LimeSurvey calls this question Q788</t>
         </is>
       </c>
     </row>
@@ -14706,7 +14706,7 @@
       </c>
       <c r="E494" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q709</t>
+          <t>LimeSurvey calls this question Q789</t>
         </is>
       </c>
     </row>
@@ -14752,7 +14752,7 @@
       </c>
       <c r="E496" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q710</t>
+          <t>LimeSurvey calls this question Q790</t>
         </is>
       </c>
     </row>
@@ -14798,7 +14798,7 @@
       </c>
       <c r="E498" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q711</t>
+          <t>LimeSurvey calls this question Q791</t>
         </is>
       </c>
     </row>
@@ -14844,7 +14844,7 @@
       </c>
       <c r="E500" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q712</t>
+          <t>LimeSurvey calls this question Q792</t>
         </is>
       </c>
     </row>
@@ -14890,7 +14890,7 @@
       </c>
       <c r="E502" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q713</t>
+          <t>LimeSurvey calls this question Q793</t>
         </is>
       </c>
     </row>
@@ -14936,7 +14936,7 @@
       </c>
       <c r="E504" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q714</t>
+          <t>LimeSurvey calls this question Q794</t>
         </is>
       </c>
     </row>
@@ -14982,7 +14982,7 @@
       </c>
       <c r="E506" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q715</t>
+          <t>LimeSurvey calls this question Q795</t>
         </is>
       </c>
     </row>
@@ -15028,7 +15028,7 @@
       </c>
       <c r="E508" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q716</t>
+          <t>LimeSurvey calls this question Q796</t>
         </is>
       </c>
     </row>
@@ -15074,7 +15074,7 @@
       </c>
       <c r="E510" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q717</t>
+          <t>LimeSurvey calls this question Q797</t>
         </is>
       </c>
     </row>
@@ -15120,7 +15120,7 @@
       </c>
       <c r="E512" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q708</t>
+          <t>LimeSurvey calls this question Q788</t>
         </is>
       </c>
     </row>
@@ -15166,7 +15166,7 @@
       </c>
       <c r="E514" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q709</t>
+          <t>LimeSurvey calls this question Q789</t>
         </is>
       </c>
     </row>
@@ -15212,7 +15212,7 @@
       </c>
       <c r="E516" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q710</t>
+          <t>LimeSurvey calls this question Q790</t>
         </is>
       </c>
     </row>
@@ -15258,7 +15258,7 @@
       </c>
       <c r="E518" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q711</t>
+          <t>LimeSurvey calls this question Q791</t>
         </is>
       </c>
     </row>
@@ -15304,7 +15304,7 @@
       </c>
       <c r="E520" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q712</t>
+          <t>LimeSurvey calls this question Q792</t>
         </is>
       </c>
     </row>
@@ -15350,7 +15350,7 @@
       </c>
       <c r="E522" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q713</t>
+          <t>LimeSurvey calls this question Q793</t>
         </is>
       </c>
     </row>
@@ -15396,7 +15396,7 @@
       </c>
       <c r="E524" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q714</t>
+          <t>LimeSurvey calls this question Q794</t>
         </is>
       </c>
     </row>
@@ -15442,7 +15442,7 @@
       </c>
       <c r="E526" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q715</t>
+          <t>LimeSurvey calls this question Q795</t>
         </is>
       </c>
     </row>
@@ -15488,7 +15488,7 @@
       </c>
       <c r="E528" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q716</t>
+          <t>LimeSurvey calls this question Q796</t>
         </is>
       </c>
     </row>
@@ -15580,7 +15580,7 @@
       </c>
       <c r="E532" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q708</t>
+          <t>LimeSurvey calls this question Q788</t>
         </is>
       </c>
     </row>
@@ -15626,7 +15626,7 @@
       </c>
       <c r="E534" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q709</t>
+          <t>LimeSurvey calls this question Q789</t>
         </is>
       </c>
     </row>
@@ -15672,7 +15672,7 @@
       </c>
       <c r="E536" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q710</t>
+          <t>LimeSurvey calls this question Q790</t>
         </is>
       </c>
     </row>
@@ -15718,7 +15718,7 @@
       </c>
       <c r="E538" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q711</t>
+          <t>LimeSurvey calls this question Q791</t>
         </is>
       </c>
     </row>
@@ -15764,7 +15764,7 @@
       </c>
       <c r="E540" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q712</t>
+          <t>LimeSurvey calls this question Q792</t>
         </is>
       </c>
     </row>
@@ -15810,7 +15810,7 @@
       </c>
       <c r="E542" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q713</t>
+          <t>LimeSurvey calls this question Q793</t>
         </is>
       </c>
     </row>
@@ -15856,7 +15856,7 @@
       </c>
       <c r="E544" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q714</t>
+          <t>LimeSurvey calls this question Q794</t>
         </is>
       </c>
     </row>
@@ -15902,7 +15902,7 @@
       </c>
       <c r="E546" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q715</t>
+          <t>LimeSurvey calls this question Q795</t>
         </is>
       </c>
     </row>
@@ -15948,7 +15948,7 @@
       </c>
       <c r="E548" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q716</t>
+          <t>LimeSurvey calls this question Q796</t>
         </is>
       </c>
     </row>
@@ -15994,7 +15994,7 @@
       </c>
       <c r="E550" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q717</t>
+          <t>LimeSurvey calls this question Q797</t>
         </is>
       </c>
     </row>
@@ -16040,7 +16040,7 @@
       </c>
       <c r="E552" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q708</t>
+          <t>LimeSurvey calls this question Q788</t>
         </is>
       </c>
     </row>
@@ -16086,7 +16086,7 @@
       </c>
       <c r="E554" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q709</t>
+          <t>LimeSurvey calls this question Q789</t>
         </is>
       </c>
     </row>
@@ -16132,7 +16132,7 @@
       </c>
       <c r="E556" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q710</t>
+          <t>LimeSurvey calls this question Q790</t>
         </is>
       </c>
     </row>
@@ -16178,7 +16178,7 @@
       </c>
       <c r="E558" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q711</t>
+          <t>LimeSurvey calls this question Q791</t>
         </is>
       </c>
     </row>
@@ -16224,7 +16224,7 @@
       </c>
       <c r="E560" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q712</t>
+          <t>LimeSurvey calls this question Q792</t>
         </is>
       </c>
     </row>
@@ -16270,7 +16270,7 @@
       </c>
       <c r="E562" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q713</t>
+          <t>LimeSurvey calls this question Q793</t>
         </is>
       </c>
     </row>
@@ -16316,7 +16316,7 @@
       </c>
       <c r="E564" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q714</t>
+          <t>LimeSurvey calls this question Q794</t>
         </is>
       </c>
     </row>
@@ -16362,7 +16362,7 @@
       </c>
       <c r="E566" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q715</t>
+          <t>LimeSurvey calls this question Q795</t>
         </is>
       </c>
     </row>
@@ -16408,7 +16408,7 @@
       </c>
       <c r="E568" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q716</t>
+          <t>LimeSurvey calls this question Q796</t>
         </is>
       </c>
     </row>
@@ -16454,7 +16454,7 @@
       </c>
       <c r="E570" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q717</t>
+          <t>LimeSurvey calls this question Q797</t>
         </is>
       </c>
     </row>
@@ -16500,7 +16500,7 @@
       </c>
       <c r="E572" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q708</t>
+          <t>LimeSurvey calls this question Q788</t>
         </is>
       </c>
     </row>
@@ -16546,7 +16546,7 @@
       </c>
       <c r="E574" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q709</t>
+          <t>LimeSurvey calls this question Q789</t>
         </is>
       </c>
     </row>
@@ -16592,7 +16592,7 @@
       </c>
       <c r="E576" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q710</t>
+          <t>LimeSurvey calls this question Q790</t>
         </is>
       </c>
     </row>
@@ -16638,7 +16638,7 @@
       </c>
       <c r="E578" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q711</t>
+          <t>LimeSurvey calls this question Q791</t>
         </is>
       </c>
     </row>
@@ -16684,7 +16684,7 @@
       </c>
       <c r="E580" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q712</t>
+          <t>LimeSurvey calls this question Q792</t>
         </is>
       </c>
     </row>
@@ -16730,7 +16730,7 @@
       </c>
       <c r="E582" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q713</t>
+          <t>LimeSurvey calls this question Q793</t>
         </is>
       </c>
     </row>
@@ -16776,7 +16776,7 @@
       </c>
       <c r="E584" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q714</t>
+          <t>LimeSurvey calls this question Q794</t>
         </is>
       </c>
     </row>
@@ -16822,7 +16822,7 @@
       </c>
       <c r="E586" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q715</t>
+          <t>LimeSurvey calls this question Q795</t>
         </is>
       </c>
     </row>
@@ -16868,7 +16868,7 @@
       </c>
       <c r="E588" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q716</t>
+          <t>LimeSurvey calls this question Q796</t>
         </is>
       </c>
     </row>
@@ -16914,7 +16914,7 @@
       </c>
       <c r="E590" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q717</t>
+          <t>LimeSurvey calls this question Q797</t>
         </is>
       </c>
     </row>
@@ -16960,7 +16960,7 @@
       </c>
       <c r="E592" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q708</t>
+          <t>LimeSurvey calls this question Q788</t>
         </is>
       </c>
     </row>
@@ -17006,7 +17006,7 @@
       </c>
       <c r="E594" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q709</t>
+          <t>LimeSurvey calls this question Q789</t>
         </is>
       </c>
     </row>
@@ -17052,7 +17052,7 @@
       </c>
       <c r="E596" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q710</t>
+          <t>LimeSurvey calls this question Q790</t>
         </is>
       </c>
     </row>
@@ -17098,7 +17098,7 @@
       </c>
       <c r="E598" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q711</t>
+          <t>LimeSurvey calls this question Q791</t>
         </is>
       </c>
     </row>
@@ -17144,7 +17144,7 @@
       </c>
       <c r="E600" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q712</t>
+          <t>LimeSurvey calls this question Q792</t>
         </is>
       </c>
     </row>
@@ -17190,7 +17190,7 @@
       </c>
       <c r="E602" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q713</t>
+          <t>LimeSurvey calls this question Q793</t>
         </is>
       </c>
     </row>
@@ -17236,7 +17236,7 @@
       </c>
       <c r="E604" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q714</t>
+          <t>LimeSurvey calls this question Q794</t>
         </is>
       </c>
     </row>
@@ -17282,7 +17282,7 @@
       </c>
       <c r="E606" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q715</t>
+          <t>LimeSurvey calls this question Q795</t>
         </is>
       </c>
     </row>
@@ -17328,7 +17328,7 @@
       </c>
       <c r="E608" s="11" t="inlineStr">
         <is>
-          <t>LimeSurvey calls this question Q716</t>
+          <t>LimeSurvey calls this question Q796</t>
         </is>
       </c>
     </row>

</xml_diff>